<commit_message>
Update MSFT data - 2026-09-06 05:42:48
</commit_message>
<xml_diff>
--- a/data/MSFT_data.xlsx
+++ b/data/MSFT_data.xlsx
@@ -5047,7 +5047,7 @@
         <v>1.108</v>
       </c>
       <c r="Q2" t="n">
-        <v>0.71</v>
+        <v>0.73</v>
       </c>
       <c r="R2" t="inlineStr">
         <is>
@@ -5093,7 +5093,7 @@
       </c>
       <c r="AB2" t="inlineStr">
         <is>
-          <t>2026-09-06 05:34:38</t>
+          <t>2026-09-06 05:41:38</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update MSFT data - 2026-09-06 16:10:47
</commit_message>
<xml_diff>
--- a/data/MSFT_data.xlsx
+++ b/data/MSFT_data.xlsx
@@ -4848,7 +4848,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB2"/>
+  <dimension ref="A1:AF2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4969,25 +4969,45 @@
       </c>
       <c r="X1" t="inlineStr">
         <is>
+          <t>book_value</t>
+        </is>
+      </c>
+      <c r="Y1" t="inlineStr">
+        <is>
+          <t>price_to_book</t>
+        </is>
+      </c>
+      <c r="Z1" t="inlineStr">
+        <is>
+          <t>earnings_growth</t>
+        </is>
+      </c>
+      <c r="AA1" t="inlineStr">
+        <is>
+          <t>shares_outstanding</t>
+        </is>
+      </c>
+      <c r="AB1" t="inlineStr">
+        <is>
           <t>sector</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="AC1" t="inlineStr">
         <is>
           <t>industry</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="AD1" t="inlineStr">
         <is>
           <t>website</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AE1" t="inlineStr">
         <is>
           <t>description</t>
         </is>
       </c>
-      <c r="AB1" t="inlineStr">
+      <c r="AF1" t="inlineStr">
         <is>
           <t>last_updated</t>
         </is>
@@ -5029,13 +5049,13 @@
         <v>3710545297408</v>
       </c>
       <c r="K2" t="n">
-        <v>28.408188</v>
+        <v>27.853958</v>
       </c>
       <c r="L2" t="n">
         <v>21.19773</v>
       </c>
       <c r="M2" t="n">
-        <v>17.59</v>
+        <v>17.94</v>
       </c>
       <c r="N2" t="n">
         <v>553.72</v>
@@ -5071,29 +5091,41 @@
       <c r="W2" t="n">
         <v>1.23</v>
       </c>
-      <c r="X2" t="inlineStr">
+      <c r="X2" t="n">
+        <v>59.565</v>
+      </c>
+      <c r="Y2" t="n">
+        <v>8.389155000000001</v>
+      </c>
+      <c r="Z2" t="n">
+        <v>0.317</v>
+      </c>
+      <c r="AA2" t="n">
+        <v>7425545491</v>
+      </c>
+      <c r="AB2" t="inlineStr">
         <is>
           <t>Technology</t>
         </is>
       </c>
-      <c r="Y2" t="inlineStr">
+      <c r="AC2" t="inlineStr">
         <is>
           <t>Software - Infrastructure</t>
         </is>
       </c>
-      <c r="Z2" t="inlineStr">
+      <c r="AD2" t="inlineStr">
         <is>
           <t>https://www.microsoft.com</t>
         </is>
       </c>
-      <c r="AA2" t="inlineStr">
+      <c r="AE2" t="inlineStr">
         <is>
           <t>Microsoft Corporation, a technology company, develops and supports a portfolio of technology solutions for individuals and businesses worldwide. Its products include operating systems, server applications, business solution applications, software development tools, desktop and server management tools, and video games; and devices, such as PCs, tablets, gaming and entertainment consoles, other intelligent devices, and related accessories. The company's Productivity and Business Processes segment offers Microsoft 365 Commercial, Enterprise Mobility + Security, Power BI, Exchange, SharePoint, Microsoft Teams, Microsoft 365 Security and Compliance, Microsoft 365 Copilot, and Windows Commercial on-premises and Office licensed on-premises. This segment also provides Microsoft 365 Consumer products and cloud services; LinkedIn, including talent solutions, marketing solutions, subscriptions, and sales solutions; Dynamics 365, a set of cloud-based applications; and on-premises ERP and CRM applications. Its Intelligent Cloud segment offers server products and cloud services; cloud and AI consumption-based services, GitHub cloud services, health and life sciences cloud services, as well as virtual desktop offerings, and other cloud services; SQL Server, Windows Server, Visual Studio, System Center, and related client access licenses; and enterprise support services, industry solutions, Microsoft partner network, and learning experience. The company's More Personal Computing segment provides Windows OEM licensing and devices comprising Surface and PC accessories; XBOX hardware, and XBOX first- and third-party content and services; XBOX Game Pass and other subscriptions; XBOX Cloud Gaming, advertising, and other cloud services; and search advertising consisting of Bing, Copilot, Microsoft News, Microsoft Edge, and third-party affiliates. It sells its products through partners and retail networks. The company was founded in 1975 and is headquartered in Redmond, Washington.</t>
         </is>
       </c>
-      <c r="AB2" t="inlineStr">
-        <is>
-          <t>2026-09-06 05:41:38</t>
+      <c r="AF2" t="inlineStr">
+        <is>
+          <t>2026-09-06 16:09:41</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update MSFT data - 2026-09-06 17:00:22
</commit_message>
<xml_diff>
--- a/data/MSFT_data.xlsx
+++ b/data/MSFT_data.xlsx
@@ -5069,15 +5069,11 @@
       <c r="Q2" t="n">
         <v>0.73</v>
       </c>
-      <c r="R2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="S2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
+      <c r="R2" t="n">
+        <v>0.40305</v>
+      </c>
+      <c r="S2" t="n">
+        <v>0.45111</v>
       </c>
       <c r="T2" t="n">
         <v>0.34039003</v>
@@ -5125,7 +5121,7 @@
       </c>
       <c r="AF2" t="inlineStr">
         <is>
-          <t>2026-09-06 16:48:46</t>
+          <t>2026-09-06 16:59:16</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update MSFT data - 2026-09-06 22:21:27
</commit_message>
<xml_diff>
--- a/data/MSFT_data.xlsx
+++ b/data/MSFT_data.xlsx
@@ -4848,7 +4848,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AF2"/>
+  <dimension ref="A1:AI2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4989,25 +4989,40 @@
       </c>
       <c r="AB1" t="inlineStr">
         <is>
+          <t>total_revenue</t>
+        </is>
+      </c>
+      <c r="AC1" t="inlineStr">
+        <is>
+          <t>enterprise_value</t>
+        </is>
+      </c>
+      <c r="AD1" t="inlineStr">
+        <is>
+          <t>ebitda</t>
+        </is>
+      </c>
+      <c r="AE1" t="inlineStr">
+        <is>
           <t>sector</t>
         </is>
       </c>
-      <c r="AC1" t="inlineStr">
+      <c r="AF1" t="inlineStr">
         <is>
           <t>industry</t>
         </is>
       </c>
-      <c r="AD1" t="inlineStr">
+      <c r="AG1" t="inlineStr">
         <is>
           <t>website</t>
         </is>
       </c>
-      <c r="AE1" t="inlineStr">
+      <c r="AH1" t="inlineStr">
         <is>
           <t>description</t>
         </is>
       </c>
-      <c r="AF1" t="inlineStr">
+      <c r="AI1" t="inlineStr">
         <is>
           <t>last_updated</t>
         </is>
@@ -5099,29 +5114,38 @@
       <c r="AA2" t="n">
         <v>7425545491</v>
       </c>
-      <c r="AB2" t="inlineStr">
+      <c r="AB2" t="n">
+        <v>331839012864</v>
+      </c>
+      <c r="AC2" t="n">
+        <v>3762515083264</v>
+      </c>
+      <c r="AD2" t="n">
+        <v>194237005824</v>
+      </c>
+      <c r="AE2" t="inlineStr">
         <is>
           <t>Technology</t>
         </is>
       </c>
-      <c r="AC2" t="inlineStr">
+      <c r="AF2" t="inlineStr">
         <is>
           <t>Software - Infrastructure</t>
         </is>
       </c>
-      <c r="AD2" t="inlineStr">
+      <c r="AG2" t="inlineStr">
         <is>
           <t>https://www.microsoft.com</t>
         </is>
       </c>
-      <c r="AE2" t="inlineStr">
+      <c r="AH2" t="inlineStr">
         <is>
           <t>Microsoft Corporation, a technology company, develops and supports a portfolio of technology solutions for individuals and businesses worldwide. Its products include operating systems, server applications, business solution applications, software development tools, desktop and server management tools, and video games; and devices, such as PCs, tablets, gaming and entertainment consoles, other intelligent devices, and related accessories. The company's Productivity and Business Processes segment offers Microsoft 365 Commercial, Enterprise Mobility + Security, Power BI, Exchange, SharePoint, Microsoft Teams, Microsoft 365 Security and Compliance, Microsoft 365 Copilot, and Windows Commercial on-premises and Office licensed on-premises. This segment also provides Microsoft 365 Consumer products and cloud services; LinkedIn, including talent solutions, marketing solutions, subscriptions, and sales solutions; Dynamics 365, a set of cloud-based applications; and on-premises ERP and CRM applications. Its Intelligent Cloud segment offers server products and cloud services; cloud and AI consumption-based services, GitHub cloud services, health and life sciences cloud services, as well as virtual desktop offerings, and other cloud services; SQL Server, Windows Server, Visual Studio, System Center, and related client access licenses; and enterprise support services, industry solutions, Microsoft partner network, and learning experience. The company's More Personal Computing segment provides Windows OEM licensing and devices comprising Surface and PC accessories; XBOX hardware, and XBOX first- and third-party content and services; XBOX Game Pass and other subscriptions; XBOX Cloud Gaming, advertising, and other cloud services; and search advertising consisting of Bing, Copilot, Microsoft News, Microsoft Edge, and third-party affiliates. It sells its products through partners and retail networks. The company was founded in 1975 and is headquartered in Redmond, Washington.</t>
         </is>
       </c>
-      <c r="AF2" t="inlineStr">
-        <is>
-          <t>2026-09-06 16:59:16</t>
+      <c r="AI2" t="inlineStr">
+        <is>
+          <t>2026-09-06 22:20:21</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update MSFT data - 2026-09-08 08:53:13
</commit_message>
<xml_diff>
--- a/data/MSFT_data.xlsx
+++ b/data/MSFT_data.xlsx
@@ -472,16 +472,16 @@
         <v>45905</v>
       </c>
       <c r="B2" t="n">
-        <v>504.9157608525771</v>
+        <v>504.9157294675595</v>
       </c>
       <c r="C2" t="n">
-        <v>507.7920894589463</v>
+        <v>507.7920578951392</v>
       </c>
       <c r="D2" t="n">
-        <v>488.3520284612672</v>
+        <v>488.3519981058333</v>
       </c>
       <c r="E2" t="n">
-        <v>490.9605712890625</v>
+        <v>490.9605407714844</v>
       </c>
       <c r="F2" t="n">
         <v>31994800</v>
@@ -498,16 +498,16 @@
         <v>45908</v>
       </c>
       <c r="B3" t="n">
-        <v>494.0451377441344</v>
+        <v>494.0451682561979</v>
       </c>
       <c r="C3" t="n">
-        <v>497.1099483047291</v>
+        <v>497.1099790060742</v>
       </c>
       <c r="D3" t="n">
-        <v>490.990285532587</v>
+        <v>490.9903158559839</v>
       </c>
       <c r="E3" t="n">
-        <v>494.1344299316406</v>
+        <v>494.1344604492188</v>
       </c>
       <c r="F3" t="n">
         <v>16771000</v>
@@ -550,16 +550,16 @@
         <v>45910</v>
       </c>
       <c r="B5" t="n">
-        <v>498.8754600894228</v>
+        <v>498.8754294126598</v>
       </c>
       <c r="C5" t="n">
-        <v>499.1234199731124</v>
+        <v>499.1233892811019</v>
       </c>
       <c r="D5" t="n">
-        <v>492.6665349159027</v>
+        <v>492.6665046209378</v>
       </c>
       <c r="E5" t="n">
-        <v>496.2867431640625</v>
+        <v>496.2867126464844</v>
       </c>
       <c r="F5" t="n">
         <v>21611800</v>
@@ -576,16 +576,16 @@
         <v>45911</v>
       </c>
       <c r="B6" t="n">
-        <v>498.1513800613702</v>
+        <v>498.1514106544788</v>
       </c>
       <c r="C6" t="n">
-        <v>499.0638857033828</v>
+        <v>499.0639163525314</v>
       </c>
       <c r="D6" t="n">
-        <v>493.8170463660224</v>
+        <v>493.8170766929454</v>
       </c>
       <c r="E6" t="n">
-        <v>496.9215087890625</v>
+        <v>496.9215393066406</v>
       </c>
       <c r="F6" t="n">
         <v>18881600</v>
@@ -628,16 +628,16 @@
         <v>45915</v>
       </c>
       <c r="B8" t="n">
-        <v>504.6379958107742</v>
+        <v>504.6380560678344</v>
       </c>
       <c r="C8" t="n">
-        <v>511.2634457193681</v>
+        <v>511.2635067675502</v>
       </c>
       <c r="D8" t="n">
-        <v>502.8625947427051</v>
+        <v>502.8626547877709</v>
       </c>
       <c r="E8" t="n">
-        <v>511.1543579101562</v>
+        <v>511.1544189453125</v>
       </c>
       <c r="F8" t="n">
         <v>17143800</v>
@@ -706,16 +706,16 @@
         <v>45918</v>
       </c>
       <c r="B11" t="n">
-        <v>507.3159513893766</v>
+        <v>507.3159820894167</v>
       </c>
       <c r="C11" t="n">
-        <v>508.883074673213</v>
+        <v>508.883105468087</v>
       </c>
       <c r="D11" t="n">
-        <v>503.5172196080818</v>
+        <v>503.517250078243</v>
       </c>
       <c r="E11" t="n">
-        <v>504.30078125</v>
+        <v>504.3008117675781</v>
       </c>
       <c r="F11" t="n">
         <v>18913700</v>
@@ -732,16 +732,16 @@
         <v>45919</v>
       </c>
       <c r="B12" t="n">
-        <v>506.3935778296786</v>
+        <v>506.3935176630351</v>
       </c>
       <c r="C12" t="n">
-        <v>515.0622454615835</v>
+        <v>515.0621842649809</v>
       </c>
       <c r="D12" t="n">
-        <v>506.1456179521661</v>
+        <v>506.1455578149837</v>
       </c>
       <c r="E12" t="n">
-        <v>513.7034301757812</v>
+        <v>513.703369140625</v>
       </c>
       <c r="F12" t="n">
         <v>52474100</v>
@@ -810,16 +810,16 @@
         <v>45924</v>
       </c>
       <c r="B15" t="n">
-        <v>506.2150114062044</v>
+        <v>506.215041937542</v>
       </c>
       <c r="C15" t="n">
-        <v>508.297849987297</v>
+        <v>508.2978806442567</v>
       </c>
       <c r="D15" t="n">
-        <v>502.7832554652563</v>
+        <v>502.7832857896144</v>
       </c>
       <c r="E15" t="n">
-        <v>505.9868774414062</v>
+        <v>505.9869079589844</v>
       </c>
       <c r="F15" t="n">
         <v>13533700</v>
@@ -862,16 +862,16 @@
         <v>45926</v>
       </c>
       <c r="B17" t="n">
-        <v>505.8976246789574</v>
+        <v>505.8975942449135</v>
       </c>
       <c r="C17" t="n">
-        <v>509.7459665668783</v>
+        <v>509.745935901324</v>
       </c>
       <c r="D17" t="n">
-        <v>502.4856945681329</v>
+        <v>502.4856643393456</v>
       </c>
       <c r="E17" t="n">
-        <v>507.2861938476562</v>
+        <v>507.2861633300781</v>
       </c>
       <c r="F17" t="n">
         <v>16213100</v>
@@ -888,16 +888,16 @@
         <v>45929</v>
       </c>
       <c r="B18" t="n">
-        <v>507.3258652143003</v>
+        <v>507.325895548039</v>
       </c>
       <c r="C18" t="n">
-        <v>512.6321819161793</v>
+        <v>512.6322125671903</v>
       </c>
       <c r="D18" t="n">
-        <v>504.7272507672145</v>
+        <v>504.7272809455783</v>
       </c>
       <c r="E18" t="n">
-        <v>510.4005432128906</v>
+        <v>510.4005737304688</v>
       </c>
       <c r="F18" t="n">
         <v>17617800</v>
@@ -940,16 +940,16 @@
         <v>45931</v>
       </c>
       <c r="B20" t="n">
-        <v>510.5989067561486</v>
+        <v>510.5989672146665</v>
       </c>
       <c r="C20" t="n">
-        <v>516.2623314762835</v>
+        <v>516.262392605391</v>
       </c>
       <c r="D20" t="n">
-        <v>507.5143007767599</v>
+        <v>507.5143608700387</v>
       </c>
       <c r="E20" t="n">
-        <v>515.4688720703125</v>
+        <v>515.4689331054688</v>
       </c>
       <c r="F20" t="n">
         <v>22632300</v>
@@ -1044,16 +1044,16 @@
         <v>45937</v>
       </c>
       <c r="B24" t="n">
-        <v>523.9788663400786</v>
+        <v>523.9788048028778</v>
       </c>
       <c r="C24" t="n">
-        <v>525.4765536672338</v>
+        <v>525.4764919541412</v>
       </c>
       <c r="D24" t="n">
-        <v>517.1847899970462</v>
+        <v>517.1847292577561</v>
       </c>
       <c r="E24" t="n">
-        <v>519.7040405273438</v>
+        <v>519.7039794921875</v>
       </c>
       <c r="F24" t="n">
         <v>14615200</v>
@@ -1096,16 +1096,16 @@
         <v>45939</v>
       </c>
       <c r="B26" t="n">
-        <v>518.0773939158137</v>
+        <v>518.07745494396</v>
       </c>
       <c r="C26" t="n">
-        <v>520.0511445409561</v>
+        <v>520.0512058016051</v>
       </c>
       <c r="D26" t="n">
-        <v>513.1777050939771</v>
+        <v>513.1777655449532</v>
       </c>
       <c r="E26" t="n">
-        <v>518.1369018554688</v>
+        <v>518.136962890625</v>
       </c>
       <c r="F26" t="n">
         <v>18343600</v>
@@ -1148,16 +1148,16 @@
         <v>45943</v>
       </c>
       <c r="B28" t="n">
-        <v>512.1958293204747</v>
+        <v>512.1957986627914</v>
       </c>
       <c r="C28" t="n">
-        <v>512.1958293204747</v>
+        <v>512.1957986627914</v>
       </c>
       <c r="D28" t="n">
-        <v>507.5044476763347</v>
+        <v>507.504417299456</v>
       </c>
       <c r="E28" t="n">
-        <v>509.8551025390625</v>
+        <v>509.8550720214844</v>
       </c>
       <c r="F28" t="n">
         <v>14284200</v>
@@ -1174,16 +1174,16 @@
         <v>45944</v>
       </c>
       <c r="B29" t="n">
-        <v>506.0661970064178</v>
+        <v>506.0662879637401</v>
       </c>
       <c r="C29" t="n">
-        <v>511.0750038311887</v>
+        <v>511.0750956887641</v>
       </c>
       <c r="D29" t="n">
-        <v>501.8707057043513</v>
+        <v>501.870795907601</v>
       </c>
       <c r="E29" t="n">
-        <v>509.3789367675781</v>
+        <v>509.3790283203125</v>
       </c>
       <c r="F29" t="n">
         <v>14684300</v>
@@ -1200,16 +1200,16 @@
         <v>45945</v>
       </c>
       <c r="B30" t="n">
-        <v>510.7576863019565</v>
+        <v>510.7576556934355</v>
       </c>
       <c r="C30" t="n">
-        <v>512.9694689959882</v>
+        <v>512.9694382549203</v>
       </c>
       <c r="D30" t="n">
-        <v>505.838140631098</v>
+        <v>505.838110317394</v>
       </c>
       <c r="E30" t="n">
-        <v>509.2401428222656</v>
+        <v>509.2401123046875</v>
       </c>
       <c r="F30" t="n">
         <v>14694700</v>
@@ -1226,16 +1226,16 @@
         <v>45946</v>
       </c>
       <c r="B31" t="n">
-        <v>508.3970522124076</v>
+        <v>508.3970827878481</v>
       </c>
       <c r="C31" t="n">
-        <v>512.6321652486282</v>
+        <v>512.6321960787722</v>
       </c>
       <c r="D31" t="n">
-        <v>503.983354813105</v>
+        <v>503.9833851231019</v>
       </c>
       <c r="E31" t="n">
-        <v>507.4349365234375</v>
+        <v>507.4349670410156</v>
       </c>
       <c r="F31" t="n">
         <v>15559600</v>
@@ -1252,16 +1252,16 @@
         <v>45947</v>
       </c>
       <c r="B32" t="n">
-        <v>504.8859867353243</v>
+        <v>504.8859262397143</v>
       </c>
       <c r="C32" t="n">
-        <v>511.2734052578957</v>
+        <v>511.273343996943</v>
       </c>
       <c r="D32" t="n">
-        <v>503.1700935064365</v>
+        <v>503.1700332164253</v>
       </c>
       <c r="E32" t="n">
-        <v>509.3889465332031</v>
+        <v>509.3888854980469</v>
       </c>
       <c r="F32" t="n">
         <v>19867800</v>
@@ -1278,16 +1278,16 @@
         <v>45950</v>
       </c>
       <c r="B33" t="n">
-        <v>510.4104293345006</v>
+        <v>510.4104901121901</v>
       </c>
       <c r="C33" t="n">
-        <v>514.4670788802013</v>
+        <v>514.4671401409408</v>
       </c>
       <c r="D33" t="n">
-        <v>509.2400661752128</v>
+        <v>509.2401268135401</v>
       </c>
       <c r="E33" t="n">
-        <v>512.5726318359375</v>
+        <v>512.5726928710938</v>
       </c>
       <c r="F33" t="n">
         <v>14665600</v>
@@ -1304,16 +1304,16 @@
         <v>45951</v>
       </c>
       <c r="B34" t="n">
-        <v>513.2769402267872</v>
+        <v>513.2770012430817</v>
       </c>
       <c r="C34" t="n">
-        <v>514.4572316509175</v>
+        <v>514.4572928075203</v>
       </c>
       <c r="D34" t="n">
-        <v>508.8533142722573</v>
+        <v>508.8533747626889</v>
       </c>
       <c r="E34" t="n">
-        <v>513.4356079101562</v>
+        <v>513.4356689453125</v>
       </c>
       <c r="F34" t="n">
         <v>15586200</v>
@@ -1330,16 +1330,16 @@
         <v>45952</v>
       </c>
       <c r="B35" t="n">
-        <v>516.8971212574951</v>
+        <v>516.8971823641815</v>
       </c>
       <c r="C35" t="n">
-        <v>520.9437823737373</v>
+        <v>520.943843958813</v>
       </c>
       <c r="D35" t="n">
-        <v>513.4851913413816</v>
+        <v>513.4852520447155</v>
       </c>
       <c r="E35" t="n">
-        <v>516.2920532226562</v>
+        <v>516.2921142578125</v>
       </c>
       <c r="F35" t="n">
         <v>18962700</v>
@@ -1356,16 +1356,16 @@
         <v>45953</v>
       </c>
       <c r="B36" t="n">
-        <v>518.1964698863214</v>
+        <v>518.1964086283891</v>
       </c>
       <c r="C36" t="n">
-        <v>519.6743010066873</v>
+        <v>519.6742395740552</v>
       </c>
       <c r="D36" t="n">
-        <v>514.3778516149157</v>
+        <v>514.3777908083965</v>
       </c>
       <c r="E36" t="n">
-        <v>516.3119506835938</v>
+        <v>516.3118896484375</v>
       </c>
       <c r="F36" t="n">
         <v>14023500</v>
@@ -1434,16 +1434,16 @@
         <v>45958</v>
       </c>
       <c r="B39" t="n">
-        <v>545.5116410650497</v>
+        <v>545.511702993095</v>
       </c>
       <c r="C39" t="n">
-        <v>549.2012543795508</v>
+        <v>549.2013167264516</v>
       </c>
       <c r="D39" t="n">
-        <v>536.3569832604931</v>
+        <v>536.3570441492753</v>
       </c>
       <c r="E39" t="n">
-        <v>537.6463623046875</v>
+        <v>537.6464233398438</v>
       </c>
       <c r="F39" t="n">
         <v>29986700</v>
@@ -1460,16 +1460,16 @@
         <v>45959</v>
       </c>
       <c r="B40" t="n">
-        <v>540.4929039137475</v>
+        <v>540.4929653309738</v>
       </c>
       <c r="C40" t="n">
-        <v>541.8120671168963</v>
+        <v>541.8121286840217</v>
       </c>
       <c r="D40" t="n">
-        <v>532.3498815675878</v>
+        <v>532.3499420595073</v>
       </c>
       <c r="E40" t="n">
-        <v>537.1305541992188</v>
+        <v>537.130615234375</v>
       </c>
       <c r="F40" t="n">
         <v>36023000</v>
@@ -1538,16 +1538,16 @@
         <v>45964</v>
       </c>
       <c r="B43" t="n">
-        <v>515.5680119038287</v>
+        <v>515.5680732671589</v>
       </c>
       <c r="C43" t="n">
-        <v>520.6760087890081</v>
+        <v>520.6760707602963</v>
       </c>
       <c r="D43" t="n">
-        <v>510.3906395365282</v>
+        <v>510.3907002836433</v>
       </c>
       <c r="E43" t="n">
-        <v>512.8107299804688</v>
+        <v>512.810791015625</v>
       </c>
       <c r="F43" t="n">
         <v>22374700</v>
@@ -1564,16 +1564,16 @@
         <v>45965</v>
       </c>
       <c r="B44" t="n">
-        <v>507.5838081580189</v>
+        <v>507.5837170627558</v>
       </c>
       <c r="C44" t="n">
-        <v>511.342858187808</v>
+        <v>511.3427664179142</v>
       </c>
       <c r="D44" t="n">
-        <v>503.6957838776707</v>
+        <v>503.6956934801851</v>
       </c>
       <c r="E44" t="n">
-        <v>510.1328430175781</v>
+        <v>510.1327514648438</v>
       </c>
       <c r="F44" t="n">
         <v>20958700</v>
@@ -1668,16 +1668,16 @@
         <v>45971</v>
       </c>
       <c r="B48" t="n">
-        <v>495.9594034527451</v>
+        <v>495.9593732946225</v>
       </c>
       <c r="C48" t="n">
-        <v>502.7138276367279</v>
+        <v>502.7137970678847</v>
       </c>
       <c r="D48" t="n">
-        <v>494.7295019610679</v>
+        <v>494.7294718777327</v>
       </c>
       <c r="E48" t="n">
-        <v>501.8707580566406</v>
+        <v>501.8707275390625</v>
       </c>
       <c r="F48" t="n">
         <v>26101500</v>
@@ -1772,16 +1772,16 @@
         <v>45975</v>
       </c>
       <c r="B52" t="n">
-        <v>494.1641988801248</v>
+        <v>494.164169077362</v>
       </c>
       <c r="C52" t="n">
-        <v>507.4250879884235</v>
+        <v>507.425057385904</v>
       </c>
       <c r="D52" t="n">
-        <v>493.3806372096086</v>
+        <v>493.3806074541019</v>
       </c>
       <c r="E52" t="n">
-        <v>506.0166625976562</v>
+        <v>506.0166320800781</v>
       </c>
       <c r="F52" t="n">
         <v>28505700</v>
@@ -1824,16 +1824,16 @@
         <v>45979</v>
       </c>
       <c r="B54" t="n">
-        <v>491.3275301094218</v>
+        <v>491.3274994941962</v>
       </c>
       <c r="C54" t="n">
-        <v>498.8754444722887</v>
+        <v>498.8754133867433</v>
       </c>
       <c r="D54" t="n">
-        <v>482.8076324047851</v>
+        <v>482.8076023204449</v>
       </c>
       <c r="E54" t="n">
-        <v>489.7604370117188</v>
+        <v>489.7604064941406</v>
       </c>
       <c r="F54" t="n">
         <v>33815100</v>
@@ -1902,16 +1902,16 @@
         <v>45982</v>
       </c>
       <c r="B57" t="n">
-        <v>475.4834610910571</v>
+        <v>475.4834301610789</v>
       </c>
       <c r="C57" t="n">
-        <v>475.9008266883901</v>
+        <v>475.9007957312625</v>
       </c>
       <c r="D57" t="n">
-        <v>465.31794169549</v>
+        <v>465.3179114267742</v>
       </c>
       <c r="E57" t="n">
-        <v>469.1436767578125</v>
+        <v>469.1436462402344</v>
       </c>
       <c r="F57" t="n">
         <v>31769200</v>
@@ -1954,16 +1954,16 @@
         <v>45986</v>
       </c>
       <c r="B59" t="n">
-        <v>471.0813659766461</v>
+        <v>471.0813963074052</v>
       </c>
       <c r="C59" t="n">
-        <v>476.1293271988991</v>
+        <v>476.1293578546732</v>
       </c>
       <c r="D59" t="n">
-        <v>461.9592459889855</v>
+        <v>461.9592757324133</v>
       </c>
       <c r="E59" t="n">
-        <v>473.9829406738281</v>
+        <v>473.9829711914062</v>
       </c>
       <c r="F59" t="n">
         <v>28019800</v>
@@ -1980,16 +1980,16 @@
         <v>45987</v>
       </c>
       <c r="B60" t="n">
-        <v>483.244191691805</v>
+        <v>483.244222260298</v>
       </c>
       <c r="C60" t="n">
-        <v>485.2315832491155</v>
+        <v>485.2316139433245</v>
       </c>
       <c r="D60" t="n">
-        <v>478.1664208189674</v>
+        <v>478.1664510662567</v>
       </c>
       <c r="E60" t="n">
-        <v>482.4393005371094</v>
+        <v>482.4393310546875</v>
       </c>
       <c r="F60" t="n">
         <v>25709100</v>
@@ -2084,16 +2084,16 @@
         <v>45994</v>
       </c>
       <c r="B64" t="n">
-        <v>473.3171775583083</v>
+        <v>473.3172079858148</v>
       </c>
       <c r="C64" t="n">
-        <v>481.1872310931236</v>
+        <v>481.1872620265617</v>
       </c>
       <c r="D64" t="n">
-        <v>472.2042431453193</v>
+        <v>472.2042735012802</v>
       </c>
       <c r="E64" t="n">
-        <v>474.7182922363281</v>
+        <v>474.7183227539062</v>
       </c>
       <c r="F64" t="n">
         <v>34615100</v>
@@ -2110,16 +2110,16 @@
         <v>45995</v>
       </c>
       <c r="B65" t="n">
-        <v>476.7355071807625</v>
+        <v>476.7355376297969</v>
       </c>
       <c r="C65" t="n">
-        <v>478.2856702042714</v>
+        <v>478.2857007523145</v>
       </c>
       <c r="D65" t="n">
-        <v>473.4861025034468</v>
+        <v>473.4861327449422</v>
       </c>
       <c r="E65" t="n">
-        <v>477.8086853027344</v>
+        <v>477.8087158203125</v>
       </c>
       <c r="F65" t="n">
         <v>22318200</v>
@@ -2136,16 +2136,16 @@
         <v>45996</v>
       </c>
       <c r="B66" t="n">
-        <v>479.4780643507397</v>
+        <v>479.4781253050461</v>
       </c>
       <c r="C66" t="n">
-        <v>480.3525214663767</v>
+        <v>480.3525825318497</v>
       </c>
       <c r="D66" t="n">
-        <v>475.8610275749173</v>
+        <v>475.861088069403</v>
       </c>
       <c r="E66" t="n">
-        <v>480.1140441894531</v>
+        <v>480.1141052246094</v>
       </c>
       <c r="F66" t="n">
         <v>22608700</v>
@@ -2162,16 +2162,16 @@
         <v>45999</v>
       </c>
       <c r="B67" t="n">
-        <v>481.8331998835391</v>
+        <v>481.8331697469475</v>
       </c>
       <c r="C67" t="n">
-        <v>489.1964595164875</v>
+        <v>489.1964289193556</v>
       </c>
       <c r="D67" t="n">
-        <v>481.3264052911177</v>
+        <v>481.3263751862239</v>
       </c>
       <c r="E67" t="n">
-        <v>487.9245300292969</v>
+        <v>487.9244995117188</v>
       </c>
       <c r="F67" t="n">
         <v>21965900</v>
@@ -2188,16 +2188,16 @@
         <v>46000</v>
       </c>
       <c r="B68" t="n">
-        <v>486.0166380400449</v>
+        <v>486.016607703579</v>
       </c>
       <c r="C68" t="n">
-        <v>489.0175885389743</v>
+        <v>489.0175580151932</v>
       </c>
       <c r="D68" t="n">
-        <v>485.4204144751398</v>
+        <v>485.4203841758892</v>
       </c>
       <c r="E68" t="n">
-        <v>488.918212890625</v>
+        <v>488.9181823730469</v>
       </c>
       <c r="F68" t="n">
         <v>14696100</v>
@@ -2240,16 +2240,16 @@
         <v>46002</v>
       </c>
       <c r="B70" t="n">
-        <v>473.6252433732215</v>
+        <v>473.6252734590456</v>
       </c>
       <c r="C70" t="n">
-        <v>482.9659780129214</v>
+        <v>482.9660086920916</v>
       </c>
       <c r="D70" t="n">
-        <v>472.8600781839672</v>
+        <v>472.8601082211862</v>
       </c>
       <c r="E70" t="n">
-        <v>480.422119140625</v>
+        <v>480.4221496582031</v>
       </c>
       <c r="F70" t="n">
         <v>24669200</v>
@@ -2292,16 +2292,16 @@
         <v>46006</v>
       </c>
       <c r="B72" t="n">
-        <v>477.0733729131614</v>
+        <v>477.0733420562278</v>
       </c>
       <c r="C72" t="n">
-        <v>477.6894594742654</v>
+        <v>477.6894285774835</v>
       </c>
       <c r="D72" t="n">
-        <v>469.5411415575728</v>
+        <v>469.5411111878212</v>
       </c>
       <c r="E72" t="n">
-        <v>471.82666015625</v>
+        <v>471.8266296386719</v>
       </c>
       <c r="F72" t="n">
         <v>23727700</v>
@@ -2318,16 +2318,16 @@
         <v>46007</v>
       </c>
       <c r="B73" t="n">
-        <v>468.9349812365753</v>
+        <v>468.9350114671635</v>
       </c>
       <c r="C73" t="n">
-        <v>474.8772929441188</v>
+        <v>474.8773235577871</v>
       </c>
       <c r="D73" t="n">
-        <v>467.9114757916915</v>
+        <v>467.911505956298</v>
       </c>
       <c r="E73" t="n">
-        <v>473.3867492675781</v>
+        <v>473.3867797851562</v>
       </c>
       <c r="F73" t="n">
         <v>20705600</v>
@@ -2448,16 +2448,16 @@
         <v>46014</v>
       </c>
       <c r="B78" t="n">
-        <v>481.9226163967179</v>
+        <v>481.922585996358</v>
       </c>
       <c r="C78" t="n">
-        <v>484.7546252629152</v>
+        <v>484.7545946839082</v>
       </c>
       <c r="D78" t="n">
-        <v>481.6841087754749</v>
+        <v>481.6840783901604</v>
       </c>
       <c r="E78" t="n">
-        <v>483.7808227539062</v>
+        <v>483.7807922363281</v>
       </c>
       <c r="F78" t="n">
         <v>14683600</v>
@@ -2474,16 +2474,16 @@
         <v>46015</v>
       </c>
       <c r="B79" t="n">
-        <v>482.6181758435609</v>
+        <v>482.6181454723109</v>
       </c>
       <c r="C79" t="n">
-        <v>486.0762481946253</v>
+        <v>486.0762176057581</v>
       </c>
       <c r="D79" t="n">
-        <v>481.7735283363114</v>
+        <v>481.7734980182152</v>
       </c>
       <c r="E79" t="n">
-        <v>484.9434204101562</v>
+        <v>484.9433898925781</v>
       </c>
       <c r="F79" t="n">
         <v>5855900</v>
@@ -2500,16 +2500,16 @@
         <v>46017</v>
       </c>
       <c r="B80" t="n">
-        <v>483.6417106195734</v>
+        <v>483.6416801645685</v>
       </c>
       <c r="C80" t="n">
-        <v>485.0428254417362</v>
+        <v>485.0427948985028</v>
       </c>
       <c r="D80" t="n">
-        <v>482.8964387136479</v>
+        <v>482.8964083055729</v>
       </c>
       <c r="E80" t="n">
-        <v>484.6354064941406</v>
+        <v>484.6353759765625</v>
       </c>
       <c r="F80" t="n">
         <v>8842200</v>
@@ -2578,16 +2578,16 @@
         <v>46022</v>
       </c>
       <c r="B83" t="n">
-        <v>484.7645645601486</v>
+        <v>484.7645337762783</v>
       </c>
       <c r="C83" t="n">
-        <v>485.0626915008752</v>
+        <v>485.0626606980731</v>
       </c>
       <c r="D83" t="n">
-        <v>480.253177052155</v>
+        <v>480.2531465547701</v>
       </c>
       <c r="E83" t="n">
-        <v>480.5711669921875</v>
+        <v>480.5711364746094</v>
       </c>
       <c r="F83" t="n">
         <v>15601600</v>
@@ -2630,16 +2630,16 @@
         <v>46027</v>
       </c>
       <c r="B85" t="n">
-        <v>471.071443053882</v>
+        <v>471.0714124582114</v>
       </c>
       <c r="C85" t="n">
-        <v>473.0687813775576</v>
+        <v>473.0687506521617</v>
       </c>
       <c r="D85" t="n">
-        <v>466.5401924921144</v>
+        <v>466.5401621907445</v>
       </c>
       <c r="E85" t="n">
-        <v>469.8690795898438</v>
+        <v>469.8690490722656</v>
       </c>
       <c r="F85" t="n">
         <v>25250300</v>
@@ -2682,16 +2682,16 @@
         <v>46029</v>
       </c>
       <c r="B87" t="n">
-        <v>476.7355161407656</v>
+        <v>476.7355464241618</v>
       </c>
       <c r="C87" t="n">
-        <v>486.6128550141313</v>
+        <v>486.61288592496</v>
       </c>
       <c r="D87" t="n">
-        <v>474.936929133209</v>
+        <v>474.9369593023546</v>
       </c>
       <c r="E87" t="n">
-        <v>480.422119140625</v>
+        <v>480.4221496582031</v>
       </c>
       <c r="F87" t="n">
         <v>25564200</v>
@@ -2786,16 +2786,16 @@
         <v>46035</v>
       </c>
       <c r="B91" t="n">
-        <v>471.6875193976834</v>
+        <v>471.687550175263</v>
       </c>
       <c r="C91" t="n">
-        <v>472.7805908527595</v>
+        <v>472.7806217016619</v>
       </c>
       <c r="D91" t="n">
-        <v>463.0125743921384</v>
+        <v>463.0126046036784</v>
       </c>
       <c r="E91" t="n">
-        <v>467.7028198242188</v>
+        <v>467.7028503417969</v>
       </c>
       <c r="F91" t="n">
         <v>28545800</v>
@@ -2864,16 +2864,16 @@
         <v>46038</v>
       </c>
       <c r="B94" t="n">
-        <v>454.9437666153887</v>
+        <v>454.9437362325269</v>
       </c>
       <c r="C94" t="n">
-        <v>460.2699922453042</v>
+        <v>460.2699615067369</v>
       </c>
       <c r="D94" t="n">
-        <v>453.6023014516422</v>
+        <v>453.6022711583685</v>
       </c>
       <c r="E94" t="n">
-        <v>456.9609680175781</v>
+        <v>456.9609375</v>
       </c>
       <c r="F94" t="n">
         <v>34246700</v>
@@ -2916,16 +2916,16 @@
         <v>46043</v>
       </c>
       <c r="B96" t="n">
-        <v>449.7467088388933</v>
+        <v>449.7467399398739</v>
       </c>
       <c r="C96" t="n">
-        <v>449.8361378186282</v>
+        <v>449.836168925793</v>
       </c>
       <c r="D96" t="n">
-        <v>435.9144504613163</v>
+        <v>435.9144806057656</v>
       </c>
       <c r="E96" t="n">
-        <v>441.3102111816406</v>
+        <v>441.3102416992188</v>
       </c>
       <c r="F96" t="n">
         <v>37980500</v>
@@ -3046,16 +3046,16 @@
         <v>46050</v>
       </c>
       <c r="B101" t="n">
-        <v>480.1637149068934</v>
+        <v>480.1637455245844</v>
       </c>
       <c r="C101" t="n">
-        <v>480.6903724414303</v>
+        <v>480.6904030927037</v>
       </c>
       <c r="D101" t="n">
-        <v>474.9865685400099</v>
+        <v>474.9865988275796</v>
       </c>
       <c r="E101" t="n">
-        <v>478.5936889648438</v>
+        <v>478.5937194824219</v>
       </c>
       <c r="F101" t="n">
         <v>36875400</v>
@@ -3072,16 +3072,16 @@
         <v>46051</v>
       </c>
       <c r="B102" t="n">
-        <v>437.2162272399066</v>
+        <v>437.2161962654454</v>
       </c>
       <c r="C102" t="n">
-        <v>439.7104135269112</v>
+        <v>439.7103823757502</v>
       </c>
       <c r="D102" t="n">
-        <v>418.365815756604</v>
+        <v>418.365786117595</v>
       </c>
       <c r="E102" t="n">
-        <v>430.7671508789062</v>
+        <v>430.7671203613281</v>
       </c>
       <c r="F102" t="n">
         <v>128855300</v>
@@ -3098,16 +3098,16 @@
         <v>46052</v>
       </c>
       <c r="B103" t="n">
-        <v>436.4013853645445</v>
+        <v>436.4014165119217</v>
       </c>
       <c r="C103" t="n">
-        <v>436.8286672682951</v>
+        <v>436.8286984461687</v>
       </c>
       <c r="D103" t="n">
-        <v>423.7615739365565</v>
+        <v>423.7616041817895</v>
       </c>
       <c r="E103" t="n">
-        <v>427.5773620605469</v>
+        <v>427.577392578125</v>
       </c>
       <c r="F103" t="n">
         <v>58566800</v>
@@ -3150,16 +3150,16 @@
         <v>46056</v>
       </c>
       <c r="B105" t="n">
-        <v>419.3495781995532</v>
+        <v>419.3496095186449</v>
       </c>
       <c r="C105" t="n">
-        <v>419.3893041977899</v>
+        <v>419.3893355198486</v>
       </c>
       <c r="D105" t="n">
-        <v>405.9843574339844</v>
+        <v>405.9843877548956</v>
       </c>
       <c r="E105" t="n">
-        <v>408.6176452636719</v>
+        <v>408.61767578125</v>
       </c>
       <c r="F105" t="n">
         <v>61424100</v>
@@ -3176,16 +3176,16 @@
         <v>46057</v>
       </c>
       <c r="B106" t="n">
-        <v>408.4089957411405</v>
+        <v>408.4089654586022</v>
       </c>
       <c r="C106" t="n">
-        <v>417.1535071208501</v>
+        <v>417.1534761899275</v>
       </c>
       <c r="D106" t="n">
-        <v>406.6600813351222</v>
+        <v>406.6600511822617</v>
       </c>
       <c r="E106" t="n">
-        <v>411.5788879394531</v>
+        <v>411.578857421875</v>
       </c>
       <c r="F106" t="n">
         <v>45012400</v>
@@ -3202,16 +3202,16 @@
         <v>46058</v>
       </c>
       <c r="B107" t="n">
-        <v>404.8714440282318</v>
+        <v>404.8714124431945</v>
       </c>
       <c r="C107" t="n">
-        <v>405.7260079125925</v>
+        <v>405.7259762608884</v>
       </c>
       <c r="D107" t="n">
-        <v>389.8467674620769</v>
+        <v>389.8467370491522</v>
       </c>
       <c r="E107" t="n">
-        <v>391.1882629394531</v>
+        <v>391.188232421875</v>
       </c>
       <c r="F107" t="n">
         <v>66289200</v>
@@ -3280,16 +3280,16 @@
         <v>46063</v>
       </c>
       <c r="B110" t="n">
-        <v>416.9746165751398</v>
+        <v>416.9746475616288</v>
       </c>
       <c r="C110" t="n">
-        <v>421.009018998737</v>
+        <v>421.0090502850332</v>
       </c>
       <c r="D110" t="n">
-        <v>410.0982587889407</v>
+        <v>410.0982892644293</v>
       </c>
       <c r="E110" t="n">
-        <v>410.6646423339844</v>
+        <v>410.6646728515625</v>
       </c>
       <c r="F110" t="n">
         <v>44857900</v>
@@ -3358,16 +3358,16 @@
         <v>46066</v>
       </c>
       <c r="B113" t="n">
-        <v>401.900281272875</v>
+        <v>401.900312028468</v>
       </c>
       <c r="C113" t="n">
-        <v>402.9834060634867</v>
+        <v>402.9834369019663</v>
       </c>
       <c r="D113" t="n">
-        <v>395.5406038478973</v>
+        <v>395.5406341168134</v>
       </c>
       <c r="E113" t="n">
-        <v>398.7900085449219</v>
+        <v>398.7900390625</v>
       </c>
       <c r="F113" t="n">
         <v>34091600</v>
@@ -3384,16 +3384,16 @@
         <v>46070</v>
       </c>
       <c r="B114" t="n">
-        <v>396.7032617740463</v>
+        <v>396.7032310749887</v>
       </c>
       <c r="C114" t="n">
-        <v>397.9950542597942</v>
+        <v>397.9950234607705</v>
       </c>
       <c r="D114" t="n">
-        <v>392.0428257724806</v>
+        <v>392.0427954340728</v>
       </c>
       <c r="E114" t="n">
-        <v>394.3581237792969</v>
+        <v>394.3580932617188</v>
       </c>
       <c r="F114" t="n">
         <v>32078800</v>
@@ -3410,16 +3410,16 @@
         <v>46071</v>
       </c>
       <c r="B115" t="n">
-        <v>395.6201070500213</v>
+        <v>395.6201374553349</v>
       </c>
       <c r="C115" t="n">
-        <v>400.0221720919145</v>
+        <v>400.0222028355481</v>
       </c>
       <c r="D115" t="n">
-        <v>393.8215201082963</v>
+        <v>393.8215503753798</v>
       </c>
       <c r="E115" t="n">
-        <v>397.0808410644531</v>
+        <v>397.0808715820312</v>
       </c>
       <c r="F115" t="n">
         <v>23223400</v>
@@ -11099,7 +11099,7 @@
       </c>
       <c r="AI2" t="inlineStr">
         <is>
-          <t>2026-09-07 03:08:00</t>
+          <t>2026-09-08 08:51:52</t>
         </is>
       </c>
     </row>

</xml_diff>